<commit_message>
Ajoute veille tour-operateurs, carnet de groupes Notion et prospection en lot
- radar-unseen : categorie Tour-operateur dans la veille presse (6 Google
  Alertes Asie, Moyen-Orient, USA), et radar_groupes.py qui range dans
  Notion les groupes signales par Telegram avec rappels groupes J-30/14/3.
- assistant-prospection : traitement en lot depuis un fichier Excel, trois
  types de contact (client, partenaire, agence) avec modeles FR/EN (et ZH
  pour client et partenaire), fallback "Team" sans prenom, HTML corrige
  pour que les paragraphes s'etalent normalement dans Gmail.
- a_traiter.xlsx exclu de Git : il contient des emails de prospects.
</commit_message>
<xml_diff>
--- a/radar-unseen/mots-cles.xlsx
+++ b/radar-unseen/mots-cles.xlsx
@@ -2001,7 +2001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B63"/>
+  <dimension ref="A1:B82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2026,7 +2026,6 @@
           <t>palace</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2034,7 +2033,6 @@
           <t>palaces</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2753,6 +2751,234 @@
       <c r="B63" t="inlineStr">
         <is>
           <t>Concurrent</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>tour-operateur</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>tour operator</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>agence de voyage</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>travel agency</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>voyagiste</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>dmc</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>outbound travel</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>groupe touristique</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>partenariat touristique</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>nouveau programme</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>bureau a paris</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>office in paris</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>personal shopping</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>shopping tour</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>duty free</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>vol direct</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>direct flight</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>assouplissement visa</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>visa waiver</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
         </is>
       </c>
     </row>
@@ -3073,7 +3299,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3149,6 +3375,18 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>Observer le positionnement et l'offre. Ne pas contacter</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tour-operateur</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Identifier un contact chez cette agence, proposer un partenariat commission/co-package</t>
         </is>
       </c>
     </row>
@@ -3293,7 +3531,6 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
           <t>à la fois un verbe de nomination ET un poste de cette liste.</t>
@@ -3325,7 +3562,6 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr"/>
       <c r="B6" t="inlineStr">
         <is>
           <t>Mets oui à une zone pour la promouvoir, non pour la rétrograder.</t>
@@ -3333,7 +3569,6 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
       <c r="B7" t="inlineStr">
         <is>
           <t>Colonne Variantes : toutes les orthographes possibles, séparées par des virgules.</t>
@@ -3353,7 +3588,6 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr"/>
       <c r="B9" t="inlineStr">
         <is>
           <t>quand le script n'arrive pas à deviner autrement.</t>
@@ -3373,7 +3607,6 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr"/>
       <c r="B11" t="inlineStr">
         <is>
           <t>C'est ton filtre principal contre les annonces de recrutement et la pub.</t>
@@ -3404,10 +3637,6 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
-    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -3421,7 +3650,6 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr"/>
       <c r="B16" t="inlineStr">
         <is>
           <t>Ajouter des mots-clés = plus d'articles. En retirer = moins de bruit.</t>
@@ -3429,7 +3657,6 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
       <c r="B17" t="inlineStr">
         <is>
           <t>Les accents et les majuscules n'ont aucune importance.</t>

</xml_diff>